<commit_message>
Daily EOD data and reports for 2026-08-03
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260803.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260803.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.315</v>
+        <v>1.312</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.018</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.13%</t>
+          <t>-1.35%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>201433.01</v>
+        <v>200973.47</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-2297.72</v>
+        <v>-2757.26</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.14</v>
+        <v>2.125</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.01</v>
+        <v>-0.025</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>-1.16%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>149800</v>
+        <v>148750</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-700</v>
+        <v>-1750</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.005</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-1.51%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>56308.84</v>
+        <v>56883.42</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-861.87</v>
+        <v>-287.29</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60.32</v>
+        <v>60.31</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.02%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>667440.8</v>
+        <v>667330.15</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>110.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>176.19</v>
+        <v>177.29</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-1.34</v>
+        <v>-0.24</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.75%</t>
+          <t>-0.14%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.745</v>
+        <v>0.752</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.005</v>
+        <v>0.012</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.68%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7450</v>
+        <v>7520</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>123.82</v>
+        <v>124.43</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.76</v>
+        <v>1.37</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.62%</t>
+          <t>1.11%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>495280</v>
+        <v>497720</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3040</v>
+        <v>5480</v>
       </c>
     </row>
     <row r="12">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.7</v>
+        <v>37.99</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.17</v>
+        <v>0.12</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.45%</t>
+          <t>0.32%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.25</v>
+        <v>32.415</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.7</v>
+        <v>-0.535</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-1.62%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41538</v>
+        <v>41750.52</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-901.6</v>
+        <v>-689.08</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1625754.71</v>
+        <v>1627431.62</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-2837.03</v>
+        <v>-1160.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>